<commit_message>
Align Supplementary Tables S3 and S7 data sources
</commit_message>
<xml_diff>
--- a/data/supplementary/Supplementary_Data_1.xlsx
+++ b/data/supplementary/Supplementary_Data_1.xlsx
@@ -827,7 +827,7 @@
       </c>
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>n pairs</t>
+          <t>n diseases</t>
         </is>
       </c>
       <c r="C1" s="21" t="inlineStr">
@@ -992,12 +992,12 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>43.30</t>
+          <t>43.31</t>
         </is>
       </c>
       <c r="D6" s="32" t="inlineStr">
         <is>
-          <t>39.01 to 47.00</t>
+          <t>40.28 to 45.86</t>
         </is>
       </c>
       <c r="E6" s="32" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="7">
       <c r="A7" s="32" t="inlineStr">
         <is>
-          <t>OpenSAGE vs GPT-5.5</t>
+          <t>OpenSAGE vs direct GPT-5.5</t>
         </is>
       </c>
       <c r="B7" s="32" t="inlineStr">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="C8" s="32" t="inlineStr">
         <is>
-          <t>53.15</t>
+          <t>53.16</t>
         </is>
       </c>
       <c r="D8" s="32" t="inlineStr">
         <is>
-          <t>49.05 to 56.91</t>
+          <t>47.21 to 56.98</t>
         </is>
       </c>
       <c r="E8" s="32" t="inlineStr">
@@ -1075,38 +1075,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>OpenSAGE vs pooled direct-generation comparator</t>
-        </is>
-      </c>
-      <c r="B9" s="33" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="inlineStr">
-        <is>
-          <t>42.54</t>
-        </is>
-      </c>
-      <c r="D9" s="33" t="inlineStr">
-        <is>
-          <t>39.13 to 45.61</t>
-        </is>
-      </c>
-      <c r="E9" s="33" t="inlineStr">
-        <is>
-          <t>0.00195</t>
-        </is>
-      </c>
-      <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>0.01367</t>
-        </is>
-      </c>
-    </row>
+    <row r="9"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11817,12 +11786,12 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>42.62</t>
+          <t>42.16</t>
         </is>
       </c>
       <c r="D6" s="32" t="inlineStr">
         <is>
-          <t>39.11 to 46.10</t>
+          <t>38.59 to 45.58</t>
         </is>
       </c>
       <c r="E6" s="32" t="inlineStr">
@@ -11844,12 +11813,12 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>42.67</t>
+          <t>43.42</t>
         </is>
       </c>
       <c r="D7" s="32" t="inlineStr">
         <is>
-          <t>38.80 to 45.89</t>
+          <t>40.00 to 46.24</t>
         </is>
       </c>
       <c r="E7" s="32" t="inlineStr">
@@ -11876,7 +11845,7 @@
       </c>
       <c r="D8" s="32" t="inlineStr">
         <is>
-          <t>37.98 to 45.60</t>
+          <t>38.48 to 45.15</t>
         </is>
       </c>
       <c r="E8" s="32" t="inlineStr">
@@ -11903,7 +11872,7 @@
       </c>
       <c r="D9" s="32" t="inlineStr">
         <is>
-          <t>39.12 to 45.98</t>
+          <t>38.75 to 45.92</t>
         </is>
       </c>
       <c r="E9" s="32" t="inlineStr">
@@ -11925,12 +11894,12 @@
       </c>
       <c r="C10" s="32" t="inlineStr">
         <is>
-          <t>42.15</t>
+          <t>43.45</t>
         </is>
       </c>
       <c r="D10" s="32" t="inlineStr">
         <is>
-          <t>38.57 to 45.29</t>
+          <t>40.11 to 46.25</t>
         </is>
       </c>
       <c r="E10" s="32" t="inlineStr">
@@ -11952,12 +11921,12 @@
       </c>
       <c r="C11" s="32" t="inlineStr">
         <is>
-          <t>42.49</t>
+          <t>42.84</t>
         </is>
       </c>
       <c r="D11" s="32" t="inlineStr">
         <is>
-          <t>38.68 to 45.78</t>
+          <t>38.94 to 46.05</t>
         </is>
       </c>
       <c r="E11" s="32" t="inlineStr">

</xml_diff>

<commit_message>
Harmonize final DGQC terminology and submission figures
</commit_message>
<xml_diff>
--- a/data/supplementary/Supplementary_Data_1.xlsx
+++ b/data/supplementary/Supplementary_Data_1.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Submission version: 20 July 2026</t>
+          <t>Submission version: 21 July 2026</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>All 1,512 ratings were provided by twelve expert reviewers in one blinded expert-rating round. The final DGQC score is the primary continuous endpoint; reviewer-mean DGQC and raw D1-D7 summaries derive from the same rating round.</t>
+          <t>All 1,512 ratings were provided by twelve expert reviewers in one blinded expert-rating round. The final DGQC score is the single continuous endpoint; descriptive D1-D7 means derive from the same round.</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>DGQC &gt;= 65</t>
+          <t>Final DGQC score &gt;= 65</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -746,7 +746,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>DGQC &gt;= 70</t>
+          <t>Final DGQC score &gt;= 70</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -773,7 +773,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>DGQC &gt;= 75</t>
+          <t>Final DGQC score &gt;= 75</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -808,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -1075,7 +1075,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1406,7 +1405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1533,17 +1532,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>reviewer_mean_DGQC</t>
+          <t>final_DGQC_score</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Mean weighted DGQC score calculated from the 12 reviewer ratings in the common expert-rating round.</t>
+          <t>Primary continuous endpoint reported for all Stage 1 and Stage 2 outputs from the common expert-rating round.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Released for the Stage 2 matched comparison in T002; Stage 1 reviewer-level source data remain controlled.</t>
+          <t>Released in T001 and T002.</t>
         </is>
       </c>
     </row>
@@ -1555,12 +1554,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>final_DGQC_score</t>
+          <t>expert_confirmed_CD</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Primary continuous endpoint reported for all Stage 1 and Stage 2 outputs from the common expert-rating round.</t>
+          <t>Strict dual-expert-confirmed critical-defect status.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1577,12 +1576,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>expert_confirmed_CD</t>
+          <t>expert_review_eligible</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Strict dual-expert-confirmed critical-defect status.</t>
+          <t>Final DGQC score &gt;=70 and no expert-confirmed critical defect.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1594,22 +1593,22 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>output_level_126</t>
+          <t>rating_level_1512</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>expert_review_eligible</t>
+          <t>rater_id</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Final DGQC score &gt;=70 and no expert-confirmed critical defect.</t>
+          <t>Anonymized reviewer identifier; identifiers and rating-level records are not released in the public dataset.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Released in T001 and T002.</t>
+          <t>Definition only; source dataset is controlled and is not released in this public repository.</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1620,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>rater_id</t>
+          <t>any_CD_raw</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Anonymized reviewer identifier; identifiers and rating-level records are not released in the public dataset.</t>
+          <t>Reviewer-level potential critical-defect rating coded yes/no.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1643,12 +1642,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>any_CD_raw</t>
+          <t>reviewer_DGQC_score</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Reviewer-level potential critical-defect rating coded yes/no.</t>
+          <t>Reviewer-level weighted DGQC score from the common expert-rating round.</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1665,12 +1664,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>DGQC_raw</t>
+          <t>D1-D7_ratings</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Reviewer-level weighted score.</t>
+          <t>Reviewer-level D1-D7 ratings from the common expert-rating round.</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1680,44 +1679,22 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>rating_level_1512</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>D1_raw-D7_raw</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>domain_summary</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>D1-D7_ratings</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>Reviewer-level D1-D7 ratings from the common expert-rating round.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Definition only; source dataset is controlled and is not released in this public repository.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>raw_domain_summary</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>D1_raw-D7_raw</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Mean D1-D7 ratings for Stage 1 and Stage 2 analysis subsets from the same expert-rating round.</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Aggregate means released in S12B and Supplementary Data 3; rating-level records remain controlled.</t>
         </is>
@@ -4454,7 +4431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4550,37 +4527,21 @@
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="33" t="inlineStr">
         <is>
-          <t>reviewer_mean_DGQC</t>
+          <t>Stage 1 / Stage 2</t>
         </is>
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>reviewer-mean DGQC</t>
+          <t>Stage 1 / Stage 2</t>
         </is>
       </c>
       <c r="C6" s="33" t="inlineStr">
         <is>
-          <t>Sensitivity endpoint calculated as the mean of 12 reviewer scores from the same expert-rating round.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>Stage 1 / Stage 2</t>
-        </is>
-      </c>
-      <c r="B7" s="33" t="inlineStr">
-        <is>
-          <t>Stage 1 / Stage 2</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="inlineStr">
-        <is>
           <t>Analysis-subset labels within one blinded expert-rating round.</t>
         </is>
       </c>
     </row>
+    <row r="7" ht="36" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7433,7 +7394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -7480,15 +7441,10 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Reviewer-mean DGQC</t>
+          <t>Expert-confirmed CD</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Expert-confirmed CD</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Usable draft</t>
         </is>
@@ -7527,15 +7483,10 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>71.11</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -7574,15 +7525,10 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>56.81</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7621,15 +7567,10 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>25.69</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7668,15 +7609,10 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>13.19</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7715,15 +7651,10 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>28.89</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7762,15 +7693,10 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>68.61</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7809,15 +7735,10 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>29.31</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7856,15 +7777,10 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>17.92</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7903,15 +7819,10 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>74.72</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -7950,15 +7861,10 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>64.31</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -7997,15 +7903,10 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>38.47</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8044,15 +7945,10 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>12.85</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8091,15 +7987,10 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>32.85</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8138,15 +8029,10 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>45.00</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8185,15 +8071,10 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>25.42</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8232,15 +8113,10 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>10.35</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8279,15 +8155,10 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>72.08</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -8326,15 +8197,10 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>47.01</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8373,15 +8239,10 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>32.15</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8420,15 +8281,10 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>24.86</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8467,15 +8323,10 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>22.29</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8514,15 +8365,10 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>49.03</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8561,15 +8407,10 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>28.19</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8608,15 +8449,10 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>16.94</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8655,15 +8491,10 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>74.10</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -8702,15 +8533,10 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>30.49</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8749,15 +8575,10 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>29.10</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8796,15 +8617,10 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>13.82</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8843,15 +8659,10 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8890,15 +8701,10 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>49.65</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8937,15 +8743,10 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>26.88</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8984,15 +8785,10 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>13.89</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9031,15 +8827,10 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>74.72</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -9078,15 +8869,10 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>32.36</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9125,15 +8911,10 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>26.74</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9172,15 +8953,10 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>18.54</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9219,15 +8995,10 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>38.26</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9266,15 +9037,10 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>48.19</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9313,15 +9079,10 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>24.79</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I40" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9360,15 +9121,10 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>26.25</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9407,15 +9163,10 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>64.65</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9454,15 +9205,10 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>35.28</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9501,15 +9247,10 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>27.85</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9548,15 +9289,10 @@
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>12.71</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9595,15 +9331,10 @@
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>31.04</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9642,15 +9373,10 @@
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>62.92</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9689,15 +9415,10 @@
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>38.54</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9736,15 +9457,10 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>16.46</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9783,15 +9499,10 @@
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>74.03</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -9830,15 +9541,10 @@
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>51.94</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9877,15 +9583,10 @@
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>23.61</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9924,15 +9625,10 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>17.71</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I53" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9971,15 +9667,10 @@
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>26.46</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10018,15 +9709,10 @@
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>50.69</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10065,15 +9751,10 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>28.54</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10112,15 +9793,10 @@
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>16.67</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10159,15 +9835,10 @@
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>71.74</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I58" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -10206,15 +9877,10 @@
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>58.54</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10253,15 +9919,10 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>25.69</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I60" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10300,15 +9961,10 @@
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>14.10</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I61" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10347,15 +10003,10 @@
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>25.97</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I62" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10394,15 +10045,10 @@
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>52.50</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I63" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10441,15 +10087,10 @@
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>43.68</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I64" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10488,15 +10129,10 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>17.22</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I65" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10535,15 +10171,10 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>66.81</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I66" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10582,15 +10213,10 @@
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>43.33</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I67" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10629,15 +10255,10 @@
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>27.22</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I68" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10676,15 +10297,10 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>14.79</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I69" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10723,15 +10339,10 @@
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>27.92</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I70" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10770,15 +10381,10 @@
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>63.40</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I71" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10817,15 +10423,10 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>30.28</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I72" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10864,15 +10465,10 @@
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>34.31</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -10911,15 +10507,10 @@
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>69.72</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I74" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -10958,15 +10549,10 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>53.19</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I75" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -11005,15 +10591,10 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>27.71</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I76" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -11052,15 +10633,10 @@
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>12.50</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I77" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -11099,15 +10675,10 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>28.47</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I78" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -11146,15 +10717,10 @@
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>65.07</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I79" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -11193,15 +10759,10 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>52.43</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I80" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -11240,15 +10801,10 @@
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>22.43</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I81" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -11265,7 +10821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -11398,90 +10954,6 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>0.00592</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Reviewer-mean DGQC: OpenSAGE vs direct GPT-5.5</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>15.86</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>8.91 to 22.09</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0.00195</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>7.75 to 23.98</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0.00166</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0.00592</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Reviewer-mean DGQC: OpenSAGE vs pooled direct-generation comparator</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>38.89</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>35.75 to 42.05</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0.00195</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>35.04 to 42.74</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2.82e-09</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
         <is>
           <t>0.00592</t>
         </is>
@@ -11963,17 +11435,17 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>OpenSAGE reviewer-mean DGQC</t>
+          <t>OpenSAGE final DGQC score</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Pooled comparator reviewer-mean DGQC</t>
+          <t>Pooled comparator final DGQC score</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Reviewer-mean difference</t>
+          <t>Final DGQC score difference</t>
         </is>
       </c>
     </row>
@@ -11985,17 +11457,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>71.11</t>
+          <t>72.50</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>34.35</t>
+          <t>33.55</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>36.77</t>
+          <t>38.95</t>
         </is>
       </c>
     </row>
@@ -12012,12 +11484,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>32.75</t>
+          <t>27.80</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>41.97</t>
+          <t>46.92</t>
         </is>
       </c>
     </row>
@@ -12034,12 +11506,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>31.50</t>
+          <t>28.80</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>40.59</t>
+          <t>43.28</t>
         </is>
       </c>
     </row>
@@ -12056,12 +11528,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>26.73</t>
+          <t>23.96</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>47.37</t>
+          <t>50.14</t>
         </is>
       </c>
     </row>
@@ -12078,12 +11550,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>30.73</t>
+          <t>28.76</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>43.99</t>
+          <t>45.96</t>
         </is>
       </c>
     </row>
@@ -12100,12 +11572,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>32.11</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>32.54</t>
+          <t>34.65</t>
         </is>
       </c>
     </row>
@@ -12122,12 +11594,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>30.80</t>
+          <t>25.62</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>43.22</t>
+          <t>48.41</t>
         </is>
       </c>
     </row>
@@ -12144,12 +11616,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>33.96</t>
+          <t>28.87</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>37.78</t>
+          <t>42.87</t>
         </is>
       </c>
     </row>
@@ -12166,12 +11638,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>34.46</t>
+          <t>32.45</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>32.34</t>
+          <t>34.36</t>
         </is>
       </c>
     </row>
@@ -12183,17 +11655,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>69.72</t>
+          <t>72.50</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>37.40</t>
+          <t>32.63</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>32.32</t>
+          <t>39.87</t>
         </is>
       </c>
     </row>

</xml_diff>